<commit_message>
refactor no-hole and has-hole directory and re-export
</commit_message>
<xml_diff>
--- a/experiments/results/abp/incremental/abp-sat-incremental.xlsx
+++ b/experiments/results/abp/incremental/abp-sat-incremental.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="incre_abp_x0.5" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="incre_abp_x0.5_has_hole" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="incre_abp_x0.75" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="incre_abp_x0.75_has_hole" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="incre_abp_x1" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="incre_abp_x1.25" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="incre_abp_x1.5" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="incre_abp_x0.5" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="incre_abp_x0.5_no_hole" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="incre_abp_x0.75" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="incre_abp_x0.75_no_hole" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="incre_abp_x1" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="incre_abp_x1.25" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="incre_abp_x1.5" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,13 +23,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +43,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -48,12 +51,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,67 +435,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Memory limit (MB)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Real time limit (s)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Target value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Lower bound</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Upper bound</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Highest label UNSAT</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Lowest label SAT</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Best span</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Memory consumed (MB)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Time consumed (ms)</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Optimal found</t>
         </is>
@@ -527,25 +539,25 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>16</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -610,7 +622,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>6</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -670,12 +682,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>6</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -735,12 +747,12 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>18</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -800,12 +812,12 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>9</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -865,12 +877,12 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>18</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -935,7 +947,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>18</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -995,12 +1007,12 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>18.1</t>
+          <t>13.7</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>155</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1060,12 +1072,12 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>44.3</t>
+          <t>18.9</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>199286</t>
+          <t>140</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1112,25 +1124,25 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>34</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>35</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>29.1</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>9570</t>
+          <t>64</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1190,12 +1202,12 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>66</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1255,12 +1267,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>831</t>
+          <t>76</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1312,20 +1324,20 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>188</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1185</t>
+          <t>963.2</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1805521</t>
+          <t>1806412</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -1373,20 +1385,20 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>188</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>1185.5</t>
+          <t>965.8</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1805555</t>
+          <t>1806441</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -1429,28 +1441,32 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>180</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>187</t>
+          <t>181</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>1210</t>
+          <t>443.8</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>1805193</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr"/>
+          <t>12887</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1490,28 +1506,32 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>180</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>181</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>1139.1</t>
+          <t>539.1</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>1805166</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr"/>
+          <t>21780</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1564,12 +1584,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>503.3</t>
+          <t>271.1</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>164628</t>
+          <t>1915</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1629,12 +1649,12 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>1073.1</t>
+          <t>987.6</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>173342</t>
+          <t>35501</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1681,25 +1701,25 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>259</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>131</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>259</v>
+        <v>130</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>764.9</t>
+          <t>672.1</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>323572</t>
+          <t>20464</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1746,28 +1766,32 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>168</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>169</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>241</v>
+        <v>168</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>1818.9</t>
+          <t>988</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>1805152</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr"/>
+          <t>84320</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1820,12 +1844,12 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>1075</t>
+          <t>564.6</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>82766</t>
+          <t>3028</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1872,25 +1896,25 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>327</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>328</t>
+          <t>165</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>327</v>
+        <v>164</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1362.3</t>
+          <t>942.5</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1667449</t>
+          <t>35287</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -1950,12 +1974,12 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>1390.7</t>
+          <t>688</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>113258</t>
+          <t>4068</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2002,28 +2026,32 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>290</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>293</t>
+          <t>291</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2104.7</t>
+          <t>1095.6</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>1805482</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr"/>
+          <t>58232</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2040,67 +2068,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Memory limit (MB)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Real time limit (s)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Target value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Lower bound</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Upper bound</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Highest label UNSAT</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Lowest label SAT</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Best span</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Memory consumed (MB)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Time consumed (ms)</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Optimal found</t>
         </is>
@@ -2144,25 +2172,25 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>18</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -2227,7 +2255,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>21</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -2287,12 +2315,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>26</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -2352,12 +2380,12 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>37</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -2417,12 +2445,12 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>85</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -2482,12 +2510,12 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>79</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -2552,7 +2580,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>68</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -2612,12 +2640,12 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>13.7</t>
+          <t>18.1</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>158</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -2677,12 +2705,12 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>18.9</t>
+          <t>44.3</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>199286</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -2729,25 +2757,25 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>41</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>29.1</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>9570</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -2807,12 +2835,12 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>34</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>1987</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -2872,12 +2900,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>38</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>831</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -2929,20 +2957,20 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>188</t>
+          <t>191</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>963.2</t>
+          <t>1185</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1806412</t>
+          <t>1805521</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -2990,20 +3018,20 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>188</t>
+          <t>191</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>965.8</t>
+          <t>1185.5</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1806441</t>
+          <t>1805555</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -3046,32 +3074,28 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>187</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>443.8</t>
+          <t>1210</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>12887</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1805193</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3111,32 +3135,28 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>201</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>539.1</t>
+          <t>1139.1</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>21780</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1805166</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3189,12 +3209,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>271.1</t>
+          <t>503.3</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1915</t>
+          <t>164628</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -3254,12 +3274,12 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>987.6</t>
+          <t>1073.1</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>35501</t>
+          <t>173342</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -3306,25 +3326,25 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>259</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>260</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>130</v>
+        <v>259</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>672.1</t>
+          <t>764.9</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>20464</t>
+          <t>323572</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -3371,32 +3391,28 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>168</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>242</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>168</v>
+        <v>241</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>988</t>
+          <t>1818.9</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>84320</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1805152</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3449,12 +3465,12 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>564.6</t>
+          <t>1075</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>3028</t>
+          <t>82766</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -3501,25 +3517,25 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>327</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>328</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>164</v>
+        <v>327</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>942.5</t>
+          <t>1362.3</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>35287</t>
+          <t>1667449</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -3579,12 +3595,12 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>688</t>
+          <t>1390.7</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>4068</t>
+          <t>113258</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3631,32 +3647,28 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>290</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>291</t>
+          <t>293</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>1095.6</t>
+          <t>2104.7</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>58232</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1805482</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3673,67 +3685,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Memory limit (MB)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Real time limit (s)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Target value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Lower bound</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Upper bound</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Highest label UNSAT</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Lowest label SAT</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Best span</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Memory consumed (MB)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Time consumed (ms)</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Optimal found</t>
         </is>
@@ -3777,25 +3789,25 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>11</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -3855,12 +3867,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>9</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -3920,12 +3932,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>9</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -3985,12 +3997,12 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>13.7</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>118</t>
+          <t>26</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -4050,12 +4062,12 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>12.2</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>190</t>
+          <t>15</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -4115,12 +4127,12 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>14.6</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>27</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -4180,12 +4192,12 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>17.8</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>277</t>
+          <t>28</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -4245,12 +4257,12 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>385</t>
+          <t>214</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -4297,28 +4309,32 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>51</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>52</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>103.5</t>
+          <t>27.8</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1805528</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr"/>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4358,25 +4374,25 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>52</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>53</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>44.2</t>
+          <t>24.4</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>42053</t>
+          <t>106</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -4436,12 +4452,12 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>49.2</t>
+          <t>27.7</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>50286</t>
+          <t>111</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -4501,12 +4517,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>50.5</t>
+          <t>30.3</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2707</t>
+          <t>115</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -4558,20 +4574,20 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>290</t>
+          <t>276</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>289</v>
+        <v>275</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1727.1</t>
+          <t>1404.1</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1805503</t>
+          <t>1806463</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -4619,20 +4635,20 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>290</t>
+          <t>276</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>289</v>
+        <v>275</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>1728.3</t>
+          <t>1404</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1805184</t>
+          <t>1806399</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -4675,28 +4691,32 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>270</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>307</t>
+          <t>271</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>306</v>
+        <v>270</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>1896.3</t>
+          <t>686.4</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>1805130</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr"/>
+          <t>25878</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4736,28 +4756,32 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>268</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>311</t>
+          <t>269</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>310</v>
+        <v>268</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>1608.7</t>
+          <t>801.8</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>1805163</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr"/>
+          <t>44645</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4797,30 +4821,32 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>340</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>341</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>340</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1097.4</t>
+          <t>432.8</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1804996</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr"/>
+          <t>3418</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4860,30 +4886,32 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>329</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>330</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>329</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>1755.1</t>
+          <t>1472.3</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1805243</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr"/>
+          <t>60071</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4928,25 +4956,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>195</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>1333.7</t>
+          <t>1013.6</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>1805435</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr"/>
+          <t>41804</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4986,28 +5016,32 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>252</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>425</t>
+          <t>253</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>424</v>
+        <v>252</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>1855</t>
+          <t>1507.7</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>1805494</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr"/>
+          <t>191749</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5060,12 +5094,12 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>1624.9</t>
+          <t>891.7</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>271055</t>
+          <t>4962</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -5117,25 +5151,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>247</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>246</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1915.4</t>
+          <t>1536.5</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1805256</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr"/>
+          <t>68409</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5188,12 +5224,12 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>1989</t>
+          <t>1064.6</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>299184</t>
+          <t>6863</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -5240,30 +5276,32 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>435</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>436</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>435</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>2857.6</t>
+          <t>1686.7</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>1805067</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr"/>
+          <t>124511</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5280,67 +5318,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Memory limit (MB)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Real time limit (s)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Target value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Lower bound</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Upper bound</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Highest label UNSAT</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Lowest label SAT</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Best span</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Memory consumed (MB)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Time consumed (ms)</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Optimal found</t>
         </is>
@@ -5384,25 +5422,25 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>16</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>46</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -5462,12 +5500,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>4.7</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>90</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -5527,12 +5565,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>4.6</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>72</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -5592,12 +5630,12 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>13.7</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>118</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -5657,12 +5695,12 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>12.2</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>190</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -5722,12 +5760,12 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>14.6</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>142</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -5787,12 +5825,12 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>17.8</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>277</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -5852,12 +5890,12 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>214</t>
+          <t>385</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -5904,32 +5942,28 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>58</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>27.8</t>
+          <t>103.5</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>227</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1805528</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5969,25 +6003,25 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>68</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>69</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>24.4</t>
+          <t>44.2</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>42053</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -6047,12 +6081,12 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>27.7</t>
+          <t>49.2</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>50286</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -6112,12 +6146,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>30.3</t>
+          <t>50.5</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>2707</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -6169,20 +6203,20 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>276</t>
+          <t>290</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1404.1</t>
+          <t>1727.1</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1806463</t>
+          <t>1805503</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -6230,20 +6264,20 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>276</t>
+          <t>290</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>1404</t>
+          <t>1728.3</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1806399</t>
+          <t>1805184</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -6286,32 +6320,28 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>271</t>
+          <t>307</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>270</v>
+        <v>306</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>686.4</t>
+          <t>1896.3</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>25878</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1805130</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6351,32 +6381,28 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>268</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>269</t>
+          <t>311</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>268</v>
+        <v>310</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>801.8</t>
+          <t>1608.7</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>44645</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1805163</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6416,32 +6442,30 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>340</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>341</t>
-        </is>
-      </c>
-      <c r="J18" t="n">
-        <v>340</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>432.8</t>
+          <t>1097.4</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>3418</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1804996</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6481,32 +6505,30 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>330</t>
-        </is>
-      </c>
-      <c r="J19" t="n">
-        <v>329</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>1472.3</t>
+          <t>1755.1</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>60071</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1805243</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6551,27 +6573,25 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>196</t>
-        </is>
-      </c>
-      <c r="J20" t="n">
-        <v>195</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>1013.6</t>
+          <t>1333.7</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>41804</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1805435</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6611,32 +6631,28 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>252</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>253</t>
+          <t>425</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>252</v>
+        <v>424</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>1507.7</t>
+          <t>1855</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>191749</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1805494</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6689,12 +6705,12 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>891.7</t>
+          <t>1624.9</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>4962</t>
+          <t>271055</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -6746,27 +6762,25 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>247</t>
-        </is>
-      </c>
-      <c r="J23" t="n">
-        <v>246</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1536.5</t>
+          <t>1915.4</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>68409</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1805256</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6819,12 +6833,12 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>1064.6</t>
+          <t>1989</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>6863</t>
+          <t>299184</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -6871,32 +6885,30 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>435</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>436</t>
-        </is>
-      </c>
-      <c r="J25" t="n">
-        <v>435</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>1686.7</t>
+          <t>2857.6</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>124511</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>1805067</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6913,67 +6925,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Memory limit (MB)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Real time limit (s)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Target value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Lower bound</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Upper bound</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Highest label UNSAT</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Lowest label SAT</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Best span</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Memory consumed (MB)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Time consumed (ms)</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Optimal found</t>
         </is>
@@ -8546,67 +8558,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Memory limit (MB)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Real time limit (s)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Target value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Lower bound</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Upper bound</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Highest label UNSAT</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Lowest label SAT</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Best span</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Memory consumed (MB)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Time consumed (ms)</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Optimal found</t>
         </is>
@@ -10187,67 +10199,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>File</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Memory limit (MB)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Real time limit (s)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Target value</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Lower bound</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Upper bound</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Highest label UNSAT</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Lowest label SAT</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Best span</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Memory consumed (MB)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Time consumed (ms)</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Optimal found</t>
         </is>

</xml_diff>